<commit_message>
Add legal pages and footer links across the portfolio
</commit_message>
<xml_diff>
--- a/Kundenformular.xlsx
+++ b/Kundenformular.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janhe_000\Desktop\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{655785A7-8C55-46A3-88FC-F8EDFAA2702A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3744C3C-D021-4599-A694-F48067F59E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A41D6D52-7B0F-4DAB-9C96-20F07C9C7297}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{A41D6D52-7B0F-4DAB-9C96-20F07C9C7297}"/>
   </bookViews>
   <sheets>
     <sheet name="Kundengespräch" sheetId="1" r:id="rId1"/>
     <sheet name="Aufwand - Scope" sheetId="2" r:id="rId2"/>
+    <sheet name="Preis-Modell" sheetId="4" r:id="rId3"/>
+    <sheet name="Tabelle5" sheetId="7" r:id="rId4"/>
+    <sheet name="Beispiel-Angebot" sheetId="5" r:id="rId5"/>
+    <sheet name="Beispiel-Auftrag" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="136">
   <si>
     <t>1. Projektbasis</t>
   </si>
@@ -94,9 +98,6 @@
     <t>Kontaktformular nötig?</t>
   </si>
   <si>
-    <t>CMS / pflegbare Inhalte nötig?</t>
-  </si>
-  <si>
     <t>externe Dienste nötig? (Maps, Newsletter, Social, etc.)</t>
   </si>
   <si>
@@ -154,9 +155,6 @@
     <t>Mehrsprachigkeit</t>
   </si>
   <si>
-    <t>Deployment</t>
-  </si>
-  <si>
     <t>Feedbackschleifen / Korrekturen</t>
   </si>
   <si>
@@ -194,13 +192,409 @@
   </si>
   <si>
     <t>BlaBla</t>
+  </si>
+  <si>
+    <t>Deployment / Live testen</t>
+  </si>
+  <si>
+    <t>CMS(selber pflegen können) / pflegbare Inhalte nötig?</t>
+  </si>
+  <si>
+    <t>Preis:</t>
+  </si>
+  <si>
+    <t>Stundensatz</t>
+  </si>
+  <si>
+    <t>Mein Rat für dich jetzt</t>
+  </si>
+  <si>
+    <t>Fixpreis-Rahmen, mit dem du arbeiten kannst</t>
+  </si>
+  <si>
+    <r>
+      <t>35–45 €/h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> = sehr fairer Einstieg</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>45–55 €/h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> = okay, wenn Scope klar ist und du dich sicher fühlst</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>über </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>55 €/h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> würde ich aktuell nur gehen, wenn der Auftrag sehr klar, frontend-lastig und gut eingegrenzt ist</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Standard-Einstieg: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>40 €/h</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>bei Unsicherheit oder ersten Kunden: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>35 €/h</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>bei sauberem Frontend-Redesign mit Formular und wenig Chaos: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>45 €/h</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Kleine Landingpage / Onepager: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>600–1.200 €</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Kleine Portfolio-/Business-Website mit 3–5 Seiten: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>1.500–3.000 €</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Redesign einer bestehenden kleinen Firmenwebsite: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>2.000–3.500 €</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Mit Kontaktformular, Livegang, Feinschliff, mehr Abstimmung: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>2.500–4.000 €</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Mit Mehrsprachigkeit, mehr Korrekturen, Dritttools: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>3.000–5.000 €</t>
+    </r>
+  </si>
+  <si>
+    <t>Angebot</t>
+  </si>
+  <si>
+    <t>Absender:</t>
+  </si>
+  <si>
+    <t>Empfänger:</t>
+  </si>
+  <si>
+    <t>Sanitär XYZ</t>
+  </si>
+  <si>
+    <t>z. Hd. [Name Ansprechpartner]</t>
+  </si>
+  <si>
+    <t>Jan Heß</t>
+  </si>
+  <si>
+    <t>[deine Daten]</t>
+  </si>
+  <si>
+    <t>für die Überarbeitung einer Unternehmenswebsite</t>
+  </si>
+  <si>
+    <t>Datum:</t>
+  </si>
+  <si>
+    <t>[Datum]</t>
+  </si>
+  <si>
+    <t>Betreff:</t>
+  </si>
+  <si>
+    <t>Angebot für das Redesign der bestehenden Unternehmenswebsite</t>
+  </si>
+  <si>
+    <t>Vielen Dank für das Gespräch und die Einblicke in Ihr Projekt.</t>
+  </si>
+  <si>
+    <t>Auf Basis unseres bisherigen Austauschs biete ich Ihnen die Überarbeitung Ihrer bestehenden Website in folgendem Umfang an:</t>
+  </si>
+  <si>
+    <t>Leistungsumfang:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> #=- visuelle und strukturelle Überarbeitung der bestehenden Website</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Modernisierung des Layouts und der Nutzerführung</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - responsive Umsetzung für Desktop, Tablet und Mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Überarbeitung der wichtigsten Seiten auf Basis der bestehenden Seitenstruktur</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Einbindung bzw. Überarbeitung eines Kontaktformulars</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- technischer Live-Test nach Fertigstellung</t>
+  </si>
+  <si>
+    <t>Optional bzw. bei Bedarf:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- kleinere inhaltliche Anpassungen auf Basis vorhandener Texte und Medien</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Unterstützung bei Hosting / Domain / Livegang</t>
+  </si>
+  <si>
+    <t>Nicht enthalten:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Login-Bereiche</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Datenbank-Funktionen</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- umfangreiche Backend-Entwicklung</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- CMS-Integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- größere Zusatzfunktionen außerhalb des besprochenen Scopes</t>
+  </si>
+  <si>
+    <t>Zeitlicher Rahmen:</t>
+  </si>
+  <si>
+    <t>Die Umsetzung ist nach finaler Abstimmung und Materialfreigabe innerhalb von ca. [X] Wochen realistisch.</t>
+  </si>
+  <si>
+    <t>Pauschalpreis: [XXXX] € netto / brutto</t>
+  </si>
+  <si>
+    <t>oder</t>
+  </si>
+  <si>
+    <t>Abrechnung auf Stundenbasis: [XX] € / Stunde</t>
+  </si>
+  <si>
+    <t>Zahlung:</t>
+  </si>
+  <si>
+    <t>- [z. B. 30 % Anzahlung, 70 % nach Fertigstellung]</t>
+  </si>
+  <si>
+    <t>- Zahlung nach Rechnungsstellung innerhalb von [X] Tagen</t>
+  </si>
+  <si>
+    <t>Hinweis:</t>
+  </si>
+  <si>
+    <t>Das Angebot basiert auf dem aktuell besprochenen Umfang. Zusätzliche Leistungen oder spätere Erweiterungen werden gesondert abgestimmt.</t>
+  </si>
+  <si>
+    <t>Gültigkeit:</t>
+  </si>
+  <si>
+    <t>Dieses Angebot ist gültig bis zum [Datum].</t>
+  </si>
+  <si>
+    <t>Wenn das für Sie passend klingt, freue ich mich über Ihre Rückmeldung. Im nächsten Schritt würde ich den Auftrag schriftlich zusammenfassen und den Projektstart vorbereiten.</t>
+  </si>
+  <si>
+    <t>Mit freundlichen Grüßen</t>
+  </si>
+  <si>
+    <t>Auftragsbestätigung</t>
+  </si>
+  <si>
+    <t>z. Hd. [Name]</t>
+  </si>
+  <si>
+    <t>Auftragsbestätigung für das Redesign der bestehenden Website</t>
+  </si>
+  <si>
+    <t>Hiermit bestätige ich den Auftrag zur Überarbeitung der bestehenden Unternehmenswebsite von Sanitär XYZ auf Grundlage des Angebots vom [Datum].</t>
+  </si>
+  <si>
+    <t>Beauftragter Leistungsumfang:</t>
+  </si>
+  <si>
+    <t>Vergütung:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Preis] € </t>
+  </si>
+  <si>
+    <t>[XX] € / Stunde</t>
+  </si>
+  <si>
+    <t>Geplanter Projektzeitraum: [von / bis oder ca. X Wochen]</t>
+  </si>
+  <si>
+    <t>Voraussetzungen:</t>
+  </si>
+  <si>
+    <t>- Bereitstellung aller benötigten Inhalte, Texte, Bilder und Zugänge</t>
+  </si>
+  <si>
+    <t>Zusätzliche Leistungen:</t>
+  </si>
+  <si>
+    <t>Leistungen außerhalb des oben genannten Umfangs werden gesondert abgestimmt.</t>
+  </si>
+  <si>
+    <t>Bitte bestätigen Sie den Auftrag kurz schriftlich per E-Mail, damit ich mit der weiteren Planung und Umsetzung beginnen kann.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Redesign der bestehenden Website</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- responsive Umsetzung</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Überarbeitung der bestehenden Seitenstruktur</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Einbindung / Überarbeitung des Kontaktformulars</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- technischer Abschluss- und Live-Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- zusätzliche Funktionen außerhalb des abgestimmten Scopes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =- Rückmeldungen und Freigaben innerhalb angemessener Zeit</t>
+  </si>
+  <si>
+    <t>durchschnittlicher Tagessatz für erfahrene Entwickler:</t>
+  </si>
+  <si>
+    <t>Tagessatz</t>
+  </si>
+  <si>
+    <t>Stundenlohn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+  </numFmts>
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -250,6 +644,41 @@
       <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -333,10 +762,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -363,8 +793,20 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="6" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -378,6 +820,583 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>153166</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>247932</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E53B27B4-DB99-C65C-158A-E00B8E7AD97B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="5487166" cy="2019582"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>76826</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>206</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Grafik 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15570155-2498-516F-3C2F-EE5F5202587F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5495925" y="0"/>
+          <a:ext cx="4486901" cy="1476581"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>143413</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>200218</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Grafik 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A495D9A-46CD-7EE9-DBAD-A7BA5712717C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10001250" y="0"/>
+          <a:ext cx="3858163" cy="1381318"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>257955</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>257374</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Grafik 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9FC1DA8-87E3-32BE-BF51-65DF4E1B9809}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="2371725"/>
+          <a:ext cx="5591955" cy="1428949"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>38815</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>257374</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Grafik 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF6F5EEB-44F9-C961-6191-130C634BF306}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5581650" y="2371725"/>
+          <a:ext cx="5125165" cy="1428949"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>753112</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>152586</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Grafik 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14518C7E-CB52-F3C8-6D51-C62B80FF8F92}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10668000" y="2362200"/>
+          <a:ext cx="4563112" cy="1333686"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>648322</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>9716</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Grafik 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9D7ED03-0556-9107-AD9F-3FEBBCCE19B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4248150"/>
+          <a:ext cx="4458322" cy="1371791"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>553484</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>9764</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Grafik 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3207086-9BF4-D5C1-5DD2-ADDCDA7E3BB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="5972175"/>
+          <a:ext cx="7411484" cy="1714739"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>638925</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>9762</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Grafik 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E576F4C-959C-299A-6EAF-D87B5A38D116}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7458075" y="5991225"/>
+          <a:ext cx="5372850" cy="1695687"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>324858</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>247837</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Grafik 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E0437C2-D1AA-884C-86B1-0443941F766D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12915900" y="5991225"/>
+          <a:ext cx="7220958" cy="1343212"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>696273</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>247845</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Grafik 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CFB85A0-7CC8-D9F9-0750-E9E82FB7B1B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="8001000"/>
+          <a:ext cx="6792273" cy="1400370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>524799</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>190730</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Grafik 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DAFF7A46-2869-4F67-1214-58EF3110F28B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6858000" y="7991475"/>
+          <a:ext cx="6620799" cy="1648055"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>144012</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>153081</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Grafik 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A11521B-3DDC-A44E-3C34-DA327EA59035}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15621000" y="0"/>
+          <a:ext cx="8145012" cy="4877481"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -783,72 +1802,72 @@
     </row>
     <row r="23" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -873,87 +1892,652 @@
   <sheetData>
     <row r="1" spans="1:6" s="10" customFormat="1" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="D2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="25.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A278C31C-3218-40D9-A99B-BCE84B5329B3}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="148.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="160.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.42578125" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="10" customFormat="1" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1" s="16"/>
+    </row>
+    <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="17">
+        <v>677</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="17">
+        <f>B2/8</f>
+        <v>84.625</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="25.5" x14ac:dyDescent="0.5">
+      <c r="A4" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77847E3B-6CD6-4F53-A967-585C476455C1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="16384" width="11.42578125" style="18"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{185AD57A-9967-4BE8-A20A-0B06A0B57126}">
+  <dimension ref="G1:G63"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="160.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G1" s="14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G4" s="14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G9" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G16" s="14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G22" s="14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G23" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G24" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G25" s="15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G26" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G27" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G28" s="15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G30" s="14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="34" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G34" s="14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G35" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G36" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G37" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="41" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G41" s="14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G42" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="44" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G44" s="14" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G45" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G46" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="47" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G47" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="49" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G49" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G50" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G51" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G52" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G54" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="55" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G55" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="57" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G57" s="14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="58" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G58" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="60" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G60" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="62" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G62" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="63" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G63" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FBA8CF6-4842-4143-9DFB-0EBF6323CC7D}">
+  <dimension ref="G1:G50"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="138.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="22" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="24" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G30" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="32" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="34" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="35" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G37" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G40" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G41" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="42" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G42" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G44" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="45" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G45" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G47" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="49" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G49" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="50" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G50" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restructure pages to use clean URLs and root-relative paths
</commit_message>
<xml_diff>
--- a/Kundenformular.xlsx
+++ b/Kundenformular.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janhe_000\Desktop\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3744C3C-D021-4599-A694-F48067F59E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C2E4DB-0488-4240-826A-A97605BE421E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{A41D6D52-7B0F-4DAB-9C96-20F07C9C7297}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{A41D6D52-7B0F-4DAB-9C96-20F07C9C7297}"/>
   </bookViews>
   <sheets>
     <sheet name="Kundengespräch" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Tabelle5" sheetId="7" r:id="rId4"/>
     <sheet name="Beispiel-Angebot" sheetId="5" r:id="rId5"/>
     <sheet name="Beispiel-Auftrag" sheetId="6" r:id="rId6"/>
+    <sheet name="Tabelle1" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1399,6 +1400,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>343480</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38637</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{359CC13D-CF46-B027-09A1-C3093BC7665B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="4153480" cy="3848637"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -2543,4 +2593,14 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A46B7A-EA55-429D-85F5-C57CF5A091F3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>